<commit_message>
Add pre-alpha audit specs 0068/0069 and Pre-Alpha Audit punch list tab
Spec 0068: read-only audit of deployed state vs repo (7 P0s: public
uploads bucket, co-owner and pet-sit self-grant, anon-callable server
functions, account deletion wiping shared-pet records and co-owner
access, Terms/Privacy behind login).

Spec 0069: security review of areas 0068 didn't cover (2 P0s: sitter
access never expires, password-reset delivery unverified).

Launch planner: new "Pre-Alpha Audit" tab combining both into 43 ranked
items. Existing tabs, dashboard chart and formulas unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/Wysker_Watch_Launch_Plan.xlsx
+++ b/docs/planning/Wysker_Watch_Launch_Plan.xlsx
@@ -15,7 +15,11 @@
   <sheets>
     <sheet name="Executive Dashboard" sheetId="1" r:id="rId1"/>
     <sheet name="Launch Plan" sheetId="2" r:id="rId2"/>
+    <sheet name="Pre-Alpha Audit" sheetId="3" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pre-Alpha Audit'!$A$4:$K$47</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -10414,4 +10418,2570 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K47"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="62" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="90" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="20" customHeight="1">
+      <c r="A1" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wysker Watch — Pre-Alpha Audit Punch List</t>
+        </is>
+      </c>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combined from spec 0068 (deployed-state audit) and spec 0069 (security review), 2026-10-23. P0 = fix before alpha kickoff on 2026-11-02. Each fix needs its own spec and Lynn's review before any code is written. Filter with the header dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item ID</t>
+        </is>
+      </c>
+      <c r="B4" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rank</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Area</t>
+        </is>
+      </c>
+      <c r="D4" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fix Type</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Status</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blocks Alpha?</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fix Spec</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="49" customHeight="1">
+      <c r="A5" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-01</t>
+        </is>
+      </c>
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Storage</t>
+        </is>
+      </c>
+      <c r="D5" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Make the uploads bucket private. Anyone, even logged out, can currently list and download every pet photo and scanned vet document.</t>
+        </is>
+      </c>
+      <c r="E5" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P0-1</t>
+        </is>
+      </c>
+      <c r="F5" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G5" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration + Frontend + Edge Function</t>
+        </is>
+      </c>
+      <c r="H5" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I5" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J5" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K5" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Switch to short-lived signed links (storageClient.js), store file paths instead of public URLs, add a size cap and image/PDF-only rule. ask-vet-assistant must download files server-side. Also covers 0069's note that observation photo links accept any outside URL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="49" customHeight="1">
+      <c r="A6" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-02</t>
+        </is>
+      </c>
+      <c r="B6" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Access control</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop strangers from making themselves a pet's co-owner. Any signed-in user who knows a pet's ID can add themselves, invisibly, and then edit or delete the pet.</t>
+        </is>
+      </c>
+      <c r="E6" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P0-2</t>
+        </is>
+      </c>
+      <c r="F6" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G6" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration</t>
+        </is>
+      </c>
+      <c r="H6" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I6" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J6" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K6" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Insert rule must require the caller to already own the pet, and only the invite-claim step may link a user. Let every owner of a pet see all its co-owners. Add a stranger test (test1@ on test4@'s pet must fail).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="34" customHeight="1">
+      <c r="A7" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-03</t>
+        </is>
+      </c>
+      <c r="B7" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Access control</t>
+        </is>
+      </c>
+      <c r="D7" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop strangers from giving themselves read access to any pet through a fake pet-sit.</t>
+        </is>
+      </c>
+      <c r="E7" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P0-3</t>
+        </is>
+      </c>
+      <c r="F7" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G7" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration</t>
+        </is>
+      </c>
+      <c r="H7" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I7" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J7" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K7" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pet-sit and sitter-access rules must require the caller to own every pet in the sit, not just one. Same fix spec as PA-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="49" customHeight="1">
+      <c r="A8" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-04</t>
+        </is>
+      </c>
+      <c r="B8" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Access control</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Make sitter access end when the sit ends. Today a sitter can read the pet's profile and every future check-in forever, which contradicts the Privacy Policy.</t>
+        </is>
+      </c>
+      <c r="E8" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P0-1</t>
+        </is>
+      </c>
+      <c r="F8" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G8" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration + Decision</t>
+        </is>
+      </c>
+      <c r="H8" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I8" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J8" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K8" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add the sit's date range to the sitter-access check. Decision needed from Lynn: should sitters see the pet before the sit starts, and for how long after it ends? Prod has 0 sits today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="64" customHeight="1">
+      <c r="A9" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-05</t>
+        </is>
+      </c>
+      <c r="B9" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Database functions</t>
+        </is>
+      </c>
+      <c r="D9" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lock down server-only database functions that anyone, even logged out, can call. One of them lets a stranger permanently block email to any address.</t>
+        </is>
+      </c>
+      <c r="E9" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P0-4, P1-7, P2; 0069 P2</t>
+        </is>
+      </c>
+      <c r="F9" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G9" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration + Edge Function</t>
+        </is>
+      </c>
+      <c r="H9" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I9" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J9" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K9" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revoke access from logged-out and logged-in users on every server-only function (staging is already correct, prod and dev aren't). Stop returning the email message ID to the browser. Rewrite the owner/sitter check functions to use the caller's own ID. Note: password resets are not affected by the email block (0069 correction).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="49" customHeight="1">
+      <c r="A10" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-06</t>
+        </is>
+      </c>
+      <c r="B10" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data lifecycle</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop account deletion from erasing records the person entered on a shared pet (check-ins, observations, vaccinations).</t>
+        </is>
+      </c>
+      <c r="E10" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P0-5</t>
+        </is>
+      </c>
+      <c r="F10" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G10" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration + Tests</t>
+        </is>
+      </c>
+      <c r="H10" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I10" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J10" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K10" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Change the 'entered by' links on the record tables from 'delete with the account' to 'keep the record, clear the name'. Tests must have the departing person enter real records first and confirm they survive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="49" customHeight="1">
+      <c r="A11" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-07</t>
+        </is>
+      </c>
+      <c r="B11" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data lifecycle</t>
+        </is>
+      </c>
+      <c r="D11" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fix delete-account so other co-owners keep access and the transferred pet keeps its photo and documents.</t>
+        </is>
+      </c>
+      <c r="E11" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P0-6; 0068 P2</t>
+        </is>
+      </c>
+      <c r="F11" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G11" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge Function + Tests</t>
+        </is>
+      </c>
+      <c r="H11" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I11" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J11" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K11" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share one co-owner transfer helper with delete-pet (which already does this right). Move, don't delete, files belonging to transferred pets. Handle more than 100 files. Also fix the partial-failure case and the misleading header comment. Add a 3-person test with a photo and a scanned document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="34" customHeight="1">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-08</t>
+        </is>
+      </c>
+      <c r="B12" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-run journey</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Make the Terms and Privacy pages open for signed-out visitors. The links on the signup screen currently bounce to the login page.</t>
+        </is>
+      </c>
+      <c r="E12" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P0-7</t>
+        </is>
+      </c>
+      <c r="F12" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G12" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frontend</t>
+        </is>
+      </c>
+      <c r="H12" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I12" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J12" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K12" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Move the 4 legal page routes outside the logged-in section of App.jsx. Add one Playwright test. Run design-system-check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="49" customHeight="1">
+      <c r="A13" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-09</t>
+        </is>
+      </c>
+      <c r="B13" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P0</t>
+        </is>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-run journey</t>
+        </is>
+      </c>
+      <c r="D13" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Make sure friend testers can reset a forgotten password, and that the app tells them if the reset email fails.</t>
+        </is>
+      </c>
+      <c r="E13" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P0-2</t>
+        </is>
+      </c>
+      <c r="F13" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn / Claude Code</t>
+        </is>
+      </c>
+      <c r="G13" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard check + Frontend</t>
+        </is>
+      </c>
+      <c r="H13" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I13" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="J13" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K13" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn: check Supabase &gt; prod &gt; Authentication &gt; Emails &gt; SMTP Settings. If custom SMTP is off, Supabase's built-in mailer only delivers to team addresses. Code: ForgotPassword.jsx currently always says 'sent', even when it failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="49" customHeight="1">
+      <c r="A14" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-10</t>
+        </is>
+      </c>
+      <c r="B14" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abuse &amp; cost</t>
+        </is>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add ownership checks and a rate limit to the co-owner and sitter invite emails. Any signed-in user can send branded email to any address with no limit.</t>
+        </is>
+      </c>
+      <c r="E14" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P1-1</t>
+        </is>
+      </c>
+      <c r="F14" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G14" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge Function</t>
+        </is>
+      </c>
+      <c r="H14" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I14" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J14" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K14" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check the caller owns the pet (and look up the pet name server-side). Add a per-user limit (e.g. 10 an hour). Give the same response whether or not the address has an account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="49" customHeight="1">
+      <c r="A15" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-11</t>
+        </is>
+      </c>
+      <c r="B15" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abuse &amp; cost</t>
+        </is>
+      </c>
+      <c r="D15" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Close the open AI proxy. Any signed-in user can send any prompt to Claude, and the endpoint will fetch any URL it's given.</t>
+        </is>
+      </c>
+      <c r="E15" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P1-2</t>
+        </is>
+      </c>
+      <c r="F15" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn / Claude Code</t>
+        </is>
+      </c>
+      <c r="G15" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge Function + Dashboard</t>
+        </is>
+      </c>
+      <c r="H15" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I15" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J15" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K15" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Move prompts and safety rules server-side, only accept this project's own file links with a size cap, add a daily per-user cap, and report AI failures to Sentry. Lynn: set a monthly spend limit in the Anthropic console.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="49" customHeight="1">
+      <c r="A16" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-12</t>
+        </is>
+      </c>
+      <c r="B16" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Features</t>
+        </is>
+      </c>
+      <c r="D16" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rebuild the Vet Report's Wellness Overview from daily check-ins (Vibe). It currently shows the retired 'Health Score /10' and leaves out check-ins entirely.</t>
+        </is>
+      </c>
+      <c r="E16" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P1-3</t>
+        </is>
+      </c>
+      <c r="F16" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G16" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge Function</t>
+        </is>
+      </c>
+      <c r="H16" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I16" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J16" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K16" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow the locked spec 0012 model (Vibe and symptom count kept separate). Drop the dead wellness_scores read and fix the outdated header comment. Every alpha user's report will be missing check-ins until this ships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="34" customHeight="1">
+      <c r="A17" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-13</t>
+        </is>
+      </c>
+      <c r="B17" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Legal &amp; consent</t>
+        </is>
+      </c>
+      <c r="D17" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capture Terms/Privacy consent from invited co-owners and sitters, and ask existing accounts that never gave it.</t>
+        </is>
+      </c>
+      <c r="E17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P1-4</t>
+        </is>
+      </c>
+      <c r="F17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frontend + Migration</t>
+        </is>
+      </c>
+      <c r="H17" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I17" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J17" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K17" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add a consent checkbox to the Accept Invite page, plus a one-time in-app prompt for any account with no consent on record (11 of 13 prod accounts). Make the consent fields write-once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="49" customHeight="1">
+      <c r="A18" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-14</t>
+        </is>
+      </c>
+      <c r="B18" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C18" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Legal &amp; consent</t>
+        </is>
+      </c>
+      <c r="D18" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Make deletion match the Privacy Policy's 'permanently delete all associated data'.</t>
+        </is>
+      </c>
+      <c r="E18" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P1-5</t>
+        </is>
+      </c>
+      <c r="F18" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn / Claude Code</t>
+        </is>
+      </c>
+      <c r="G18" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Policy wording + Edge Function + Backup job</t>
+        </is>
+      </c>
+      <c r="H18" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I18" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J18" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K18" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Policy should mention that backups age out. Prune deleted users' files from the R2 storage backup, delete scanned documents when a pet is deleted, remove sitter rows when the sitter deletes their account, and decide what to say about email logs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="49" customHeight="1">
+      <c r="A19" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-15</t>
+        </is>
+      </c>
+      <c r="B19" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Silent failures</t>
+        </is>
+      </c>
+      <c r="D19" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Send backend and frontend failures to Sentry, including errors on Lynn's own account.</t>
+        </is>
+      </c>
+      <c r="E19" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P1-6; 0069 repo note</t>
+        </is>
+      </c>
+      <c r="F19" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G19" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge Function + Frontend</t>
+        </is>
+      </c>
+      <c r="H19" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I19" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J19" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K19" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add a shared helper that reports and responds in one step. Report data-loading errors from the frontend. Stop filtering out the 'owner' account type. Fix the invite dialog's stuck spinner when a save fails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="34" customHeight="1">
+      <c r="A20" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-16</t>
+        </is>
+      </c>
+      <c r="B20" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C20" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process</t>
+        </is>
+      </c>
+      <c r="D20" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Commit the cross-project comparison script and run it after every migration.</t>
+        </is>
+      </c>
+      <c r="E20" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P1-7 / AC3</t>
+        </is>
+      </c>
+      <c r="F20" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G20" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tooling + Docs</t>
+        </is>
+      </c>
+      <c r="H20" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I20" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J20" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K20" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compares functions, permissions, rules, cron, buckets, triggers and columns across dev, staging and prod. Add it to the deploy checklist in 0006 Technical Standards §11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="34" customHeight="1">
+      <c r="A21" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-17</t>
+        </is>
+      </c>
+      <c r="B21" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config</t>
+        </is>
+      </c>
+      <c r="D21" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Set prod's allowed-website list (CORS_ALLOWED_ORIGINS) and settle the real domain: www.wyskerwatch.com or wyskerwatch.com.</t>
+        </is>
+      </c>
+      <c r="E21" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P1-8; 0069 docs drift</t>
+        </is>
+      </c>
+      <c r="F21" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G21" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision + Config</t>
+        </is>
+      </c>
+      <c r="H21" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I21" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J21" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K21" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Still unset on prod. Three code comments disagree about which domain is canonical. Signup will fail for anyone arriving at the other domain unless it redirects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="49" customHeight="1">
+      <c r="A22" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-18</t>
+        </is>
+      </c>
+      <c r="B22" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C22" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account security</t>
+        </is>
+      </c>
+      <c r="D22" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stop people from pre-registering an account at someone else's email address and taking it over after the real owner clicks the confirmation link.</t>
+        </is>
+      </c>
+      <c r="E22" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P1-1; 0069 P2</t>
+        </is>
+      </c>
+      <c r="F22" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G22" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frontend + Edge Function + Migration</t>
+        </is>
+      </c>
+      <c r="H22" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I22" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J22" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K22" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Have the inbox owner set the password at the confirmation step (like Accept Invite does) and sign out other sessions. Invite claims should also require a confirmed email. Decision: OK to move password entry to the confirmation step?</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="49" customHeight="1">
+      <c r="A23" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-19</t>
+        </is>
+      </c>
+      <c r="B23" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C23" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account security</t>
+        </is>
+      </c>
+      <c r="D23" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turn off Supabase's built-in public signup on all 3 projects, so every account goes through our sign-up checks (consent, rate limits, password rules).</t>
+        </is>
+      </c>
+      <c r="E23" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P1-2</t>
+        </is>
+      </c>
+      <c r="F23" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G23" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard</t>
+        </is>
+      </c>
+      <c r="H23" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I23" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J23" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K23" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cheap; worth doing before alpha. Verify on dev first that sign-up and invites still work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="34" customHeight="1">
+      <c r="A24" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-20</t>
+        </is>
+      </c>
+      <c r="B24" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C24" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-run journey</t>
+        </is>
+      </c>
+      <c r="D24" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fix the 'Continue with Google' button. Google login is switched off, so tapping it leads to an error page.</t>
+        </is>
+      </c>
+      <c r="E24" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P1-3</t>
+        </is>
+      </c>
+      <c r="F24" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn / Claude Code</t>
+        </is>
+      </c>
+      <c r="G24" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision + Dashboard or Frontend</t>
+        </is>
+      </c>
+      <c r="H24" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I24" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J24" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K24" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision: enable Google sign-in, or hide the button until it's set up (one line per page). Cheap; worth doing before alpha, since it's on the very first screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="34" customHeight="1">
+      <c r="A25" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-21</t>
+        </is>
+      </c>
+      <c r="B25" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C25" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config</t>
+        </is>
+      </c>
+      <c r="D25" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record the login check for the two ops-only functions explicitly in supabase/config.toml.</t>
+        </is>
+      </c>
+      <c r="E25" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P1-4; 0069 docs drift</t>
+        </is>
+      </c>
+      <c r="F25" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G25" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config</t>
+        </is>
+      </c>
+      <c r="H25" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I25" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J25" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K25" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not exploitable today, but their safety depends on an unrecorded default. Also fix the send-email comment about the newer key format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="34" customHeight="1">
+      <c r="A26" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-22</t>
+        </is>
+      </c>
+      <c r="B26" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C26" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process</t>
+        </is>
+      </c>
+      <c r="D26" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adopt standing security rules so future specs don't need to ask for basic safety.</t>
+        </is>
+      </c>
+      <c r="E26" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow-up from 0068 discussion</t>
+        </is>
+      </c>
+      <c r="F26" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G26" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision + Docs</t>
+        </is>
+      </c>
+      <c r="H26" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I26" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J26" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K26" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A stranger test for every new access rule or function, test data with multiple co-owners plus real records and files, and Supabase's security scanner in CI. Needs its own spec for Lynn's review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="34" customHeight="1">
+      <c r="A27" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-23</t>
+        </is>
+      </c>
+      <c r="B27" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C27" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Docs</t>
+        </is>
+      </c>
+      <c r="D27" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Correct spec 0066's 'identical across all 3 projects' result and 0068 P0-4's 'password resets' wording.</t>
+        </is>
+      </c>
+      <c r="E27" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 docs drift; 0069 docs drift</t>
+        </is>
+      </c>
+      <c r="F27" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G27" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Docs</t>
+        </is>
+      </c>
+      <c r="H27" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I27" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J27" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K27" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Function permissions differed (see PA-05). Password resets go through Supabase's own mailer, so they aren't blocked by the fake-bounce issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="49" customHeight="1">
+      <c r="A28" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-24</t>
+        </is>
+      </c>
+      <c r="B28" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C28" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Access control</t>
+        </is>
+      </c>
+      <c r="D28" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limit what co-owners can do: today any co-owner can hand the pet's primary ownership to anyone, or delete the pet directly, skipping the transfer logic.</t>
+        </is>
+      </c>
+      <c r="E28" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P2</t>
+        </is>
+      </c>
+      <c r="F28" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G28" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration</t>
+        </is>
+      </c>
+      <c r="H28" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I28" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J28" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K28" s="54"/>
+    </row>
+    <row r="29" spans="1:11" ht="34" customHeight="1">
+      <c r="A29" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-25</t>
+        </is>
+      </c>
+      <c r="B29" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C29" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Access control</t>
+        </is>
+      </c>
+      <c r="D29" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Make the 'entered by' field on new records always the person actually signed in.</t>
+        </is>
+      </c>
+      <c r="E29" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P2</t>
+        </is>
+      </c>
+      <c r="F29" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G29" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration</t>
+        </is>
+      </c>
+      <c r="H29" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I29" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J29" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K29" s="54"/>
+    </row>
+    <row r="30" spans="1:11" ht="34" customHeight="1">
+      <c r="A30" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-26</t>
+        </is>
+      </c>
+      <c r="B30" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C30" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Access control</t>
+        </is>
+      </c>
+      <c r="D30" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Make sure sitter log entries can only be attached to pets in that sit.</t>
+        </is>
+      </c>
+      <c r="E30" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P2</t>
+        </is>
+      </c>
+      <c r="F30" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G30" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration</t>
+        </is>
+      </c>
+      <c r="H30" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I30" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J30" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K30" s="54"/>
+    </row>
+    <row r="31" spans="1:11" ht="34" customHeight="1">
+      <c r="A31" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-27</t>
+        </is>
+      </c>
+      <c r="B31" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C31" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Access control</t>
+        </is>
+      </c>
+      <c r="D31" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Make profile email read-only and match sitter invites on the verified login email.</t>
+        </is>
+      </c>
+      <c r="E31" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P2</t>
+        </is>
+      </c>
+      <c r="F31" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G31" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration</t>
+        </is>
+      </c>
+      <c r="H31" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I31" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J31" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K31" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Today someone could change their profile email to another person's and see that person's sitter-invite rows (no pet data).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="34" customHeight="1">
+      <c r="A32" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-28</t>
+        </is>
+      </c>
+      <c r="B32" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C32" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Features</t>
+        </is>
+      </c>
+      <c r="D32" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Keep sitter-only pets out of owner-only flows (Scan Record matching, Edit Pet, Vet Report).</t>
+        </is>
+      </c>
+      <c r="E32" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P2</t>
+        </is>
+      </c>
+      <c r="F32" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G32" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frontend</t>
+        </is>
+      </c>
+      <c r="H32" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I32" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J32" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K32" s="54"/>
+    </row>
+    <row r="33" spans="1:11" ht="34" customHeight="1">
+      <c r="A33" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-29</t>
+        </is>
+      </c>
+      <c r="B33" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C33" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Database functions</t>
+        </is>
+      </c>
+      <c r="D33" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Set a fixed search path on 3 database functions (security-scanner warning).</t>
+        </is>
+      </c>
+      <c r="E33" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P2</t>
+        </is>
+      </c>
+      <c r="F33" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G33" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration</t>
+        </is>
+      </c>
+      <c r="H33" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I33" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J33" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K33" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">handle_new_user, classify_account_type, set_updated_at.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="29" customHeight="1">
+      <c r="A34" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-30</t>
+        </is>
+      </c>
+      <c r="B34" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C34" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account security</t>
+        </is>
+      </c>
+      <c r="D34" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Turn on leaked-password protection in Supabase Auth.</t>
+        </is>
+      </c>
+      <c r="E34" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P2</t>
+        </is>
+      </c>
+      <c r="F34" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G34" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard</t>
+        </is>
+      </c>
+      <c r="H34" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I34" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J34" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K34" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One toggle, under Authentication &gt; Attack Protection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="34" customHeight="1">
+      <c r="A35" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-31</t>
+        </is>
+      </c>
+      <c r="B35" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C35" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abuse &amp; cost</t>
+        </is>
+      </c>
+      <c r="D35" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add the CAPTCHA to Register and 'resend confirmation' to stop inbox flooding.</t>
+        </is>
+      </c>
+      <c r="E35" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P2</t>
+        </is>
+      </c>
+      <c r="F35" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G35" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frontend + Edge Function</t>
+        </is>
+      </c>
+      <c r="H35" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I35" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J35" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K35" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same Turnstile already used on /beta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="34" customHeight="1">
+      <c r="A36" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-32</t>
+        </is>
+      </c>
+      <c r="B36" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C36" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abuse &amp; cost</t>
+        </is>
+      </c>
+      <c r="D36" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check that per-visitor signup limits see the real visitor's address, not Supabase's proxy.</t>
+        </is>
+      </c>
+      <c r="E36" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P2</t>
+        </is>
+      </c>
+      <c r="F36" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G36" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investigation</t>
+        </is>
+      </c>
+      <c r="H36" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I36" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J36" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K36" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If they see the proxy, every visitor shares one limit, and signups would be refused site-wide after 20 an hour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="34" customHeight="1">
+      <c r="A37" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-33</t>
+        </is>
+      </c>
+      <c r="B37" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C37" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abuse &amp; cost</t>
+        </is>
+      </c>
+      <c r="D37" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cap analytics event writes and exclude demo accounts from the analytics summary.</t>
+        </is>
+      </c>
+      <c r="E37" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P2; 0069 P2</t>
+        </is>
+      </c>
+      <c r="F37" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G37" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Migration</t>
+        </is>
+      </c>
+      <c r="H37" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I37" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J37" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K37" s="54"/>
+    </row>
+    <row r="38" spans="1:11" ht="34" customHeight="1">
+      <c r="A38" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-34</t>
+        </is>
+      </c>
+      <c r="B38" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C38" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Silent failures</t>
+        </is>
+      </c>
+      <c r="D38" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flush Sentry before backend functions return, so events aren't dropped.</t>
+        </is>
+      </c>
+      <c r="E38" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P2</t>
+        </is>
+      </c>
+      <c r="F38" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G38" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge Function</t>
+        </is>
+      </c>
+      <c r="H38" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I38" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J38" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K38" s="54"/>
+    </row>
+    <row r="39" spans="1:11" ht="34" customHeight="1">
+      <c r="A39" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-35</t>
+        </is>
+      </c>
+      <c r="B39" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C39" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Silent failures</t>
+        </is>
+      </c>
+      <c r="D39" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Return generic error messages from backend functions instead of internal details.</t>
+        </is>
+      </c>
+      <c r="E39" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P2</t>
+        </is>
+      </c>
+      <c r="F39" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G39" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge Function</t>
+        </is>
+      </c>
+      <c r="H39" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I39" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J39" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K39" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sentry already gets the detail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="34" customHeight="1">
+      <c r="A40" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-36</t>
+        </is>
+      </c>
+      <c r="B40" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C40" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Features</t>
+        </is>
+      </c>
+      <c r="D40" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notify existing users when they're added as a co-owner. Today they get no email or notice, and only see the pet after their next login.</t>
+        </is>
+      </c>
+      <c r="E40" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P2</t>
+        </is>
+      </c>
+      <c r="F40" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G40" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edge Function + Frontend</t>
+        </is>
+      </c>
+      <c r="H40" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I40" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J40" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K40" s="54"/>
+    </row>
+    <row r="41" spans="1:11" ht="34" customHeight="1">
+      <c r="A41" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-37</t>
+        </is>
+      </c>
+      <c r="B41" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C41" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Config</t>
+        </is>
+      </c>
+      <c r="D41" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm the 'nightly-analytics-summary' job is meant to run every hour.</t>
+        </is>
+      </c>
+      <c r="E41" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 P2</t>
+        </is>
+      </c>
+      <c r="F41" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G41" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision</t>
+        </is>
+      </c>
+      <c r="H41" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I41" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J41" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K41" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It has run 336 times in 14 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="34" customHeight="1">
+      <c r="A42" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-38</t>
+        </is>
+      </c>
+      <c r="B42" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C42" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account security</t>
+        </is>
+      </c>
+      <c r="D42" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decide how far the shared demo login should reach. It's a real, writable prod session.</t>
+        </is>
+      </c>
+      <c r="E42" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 P2</t>
+        </is>
+      </c>
+      <c r="F42" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G42" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision</t>
+        </is>
+      </c>
+      <c r="H42" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I42" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J42" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K42" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Depends on who has the demo1@ password and whether it's published anywhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="34" customHeight="1">
+      <c r="A43" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-39</t>
+        </is>
+      </c>
+      <c r="B43" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C43" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code health</t>
+        </is>
+      </c>
+      <c r="D43" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Move duplicated helpers into _shared, and wire in or delete the unused password-reset email template.</t>
+        </is>
+      </c>
+      <c r="E43" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0069 repo note</t>
+        </is>
+      </c>
+      <c r="F43" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G43" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Refactor</t>
+        </is>
+      </c>
+      <c r="H43" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I43" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J43" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K43" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Helpers: getJwtRole (2 copies); getRequestIp and verifyTurnstile (3 copies).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="49" customHeight="1">
+      <c r="A44" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-40</t>
+        </is>
+      </c>
+      <c r="B44" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C44" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Docs</t>
+        </is>
+      </c>
+      <c r="D44" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fix 4 stale CLAUDE.md notes.</t>
+        </is>
+      </c>
+      <c r="E44" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 docs drift</t>
+        </is>
+      </c>
+      <c r="F44" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G44" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Docs</t>
+        </is>
+      </c>
+      <c r="H44" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I44" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J44" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K44" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start-here path doesn't exist. The e2e 'trial through 9/3' note is stale (the job has never passed). Planner file vs Execution Plan memory needs a decision. Add a note that 0052's restored public-read rule is itself a P0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="34" customHeight="1">
+      <c r="A45" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-41</t>
+        </is>
+      </c>
+      <c r="B45" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check</t>
+        </is>
+      </c>
+      <c r="C45" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard checks</t>
+        </is>
+      </c>
+      <c r="D45" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run the Supabase Auth dashboard checklist on prod, then dev and staging.</t>
+        </is>
+      </c>
+      <c r="E45" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 OQ1; 0069 OQ2</t>
+        </is>
+      </c>
+      <c r="F45" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G45" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard check</t>
+        </is>
+      </c>
+      <c r="H45" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I45" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J45" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K45" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Secure email change on; link expiry 1 hour or less; Site URL and redirect list exact (no localhost or wildcards on prod); email rate limit; refresh-token reuse detection on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="34" customHeight="1">
+      <c r="A46" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-42</t>
+        </is>
+      </c>
+      <c r="B46" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check</t>
+        </is>
+      </c>
+      <c r="C46" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard checks</t>
+        </is>
+      </c>
+      <c r="D46" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm the live production frontend on Cloudflare is the current main build (c36f7a4).</t>
+        </is>
+      </c>
+      <c r="E46" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0068 OQ2</t>
+        </is>
+      </c>
+      <c r="F46" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G46" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard check</t>
+        </is>
+      </c>
+      <c r="H46" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I46" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J46" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K46" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Promotion is manual, and I can't see it from here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="34" customHeight="1">
+      <c r="A47" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-43</t>
+        </is>
+      </c>
+      <c r="B47" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check</t>
+        </is>
+      </c>
+      <c r="C47" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard checks</t>
+        </is>
+      </c>
+      <c r="D47" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rotate the test1@/test2@ passwords that were shared in a chat, and update the matching GitHub secrets.</t>
+        </is>
+      </c>
+      <c r="E47" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0066 open question</t>
+        </is>
+      </c>
+      <c r="F47" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G47" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard</t>
+        </is>
+      </c>
+      <c r="H47" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I47" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J47" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K47" s="54"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:K47"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B5:B47">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
+      <formula>"P0"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+      <formula>"P1"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+      <formula>"P2"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5:H47">
+    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="Complete">
+      <formula>NOT(ISERROR(SEARCH("Complete",H5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="In Progress">
+      <formula>NOT(ISERROR(SEARCH("In Progress",H5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="6" operator="containsText" text="Not Started">
+      <formula>NOT(ISERROR(SEARCH("Not Started",H5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I47">
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" sqref="H5:H67">
+      <formula1>"Not Started,In Progress,Blocked,Complete,Deferred,N/A"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="B5:B67">
+      <formula1>"P0,P1,P2,Check"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I5:I67">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Track open follow-ups on the Pre-Alpha Audit punch list
Adds PA-44 to PA-49 (build spec 0067, GitHub secrets for test3@/test4@,
CI browser caching, redo closed PRs #19/#20, intermittent e2e tests,
making e2e a required check). Updates PA-17 (Lynn: www is official, the
bare domain is also reachable), PA-23 (why 0066's "identical" result
missed function permissions) and PA-43 (password rotation in progress).

Edited the sheet XML directly so the workbook's chart is preserved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/Wysker_Watch_Launch_Plan.xlsx
+++ b/docs/planning/Wysker_Watch_Launch_Plan.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Pre-Alpha Audit" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pre-Alpha Audit'!$A$4:$K$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pre-Alpha Audit'!$A$4:$K$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -10422,7 +10422,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -11484,7 +11484,7 @@
       </c>
       <c r="K21" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Still unset on prod. Three code comments disagree about which domain is canonical. Signup will fail for anyone arriving at the other domain unless it redirects.</t>
+          <t xml:space="preserve">Still unset on prod. Three code comments disagree about which domain is canonical. Signup will fail for anyone arriving at the other domain unless it redirects. Lynn, 2026-10-24: www.wyskerwatch.com is the official address; wyskerwatch.com (no www) is also reachable and listed in Cloudflare. So: set CORS_ALLOWED_ORIGINS on prod to both, or add a Cloudflare redirect from the bare domain to www. Couldn't check from here whether a redirect already exists (Bot Fight Mode blocks automated requests).</t>
         </is>
       </c>
     </row>
@@ -11826,7 +11826,7 @@
       </c>
       <c r="K27" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Function permissions differed (see PA-05). Password resets go through Supabase's own mailer, so they aren't blocked by the fake-bounce issue.</t>
+          <t xml:space="preserve">Function permissions differed (see PA-05). Password resets go through Supabase's own mailer, so they aren't blocked by the fake-bounce issue. PR #22 (merged 2026-10-24) still carries the 'identical' wording in 0066's Results. Root cause: 0066's step-0 check compared function code and security settings, but not who may run each function.</t>
         </is>
       </c>
     </row>
@@ -12936,15 +12936,361 @@
           <t xml:space="preserve">Not written</t>
         </is>
       </c>
-      <c r="K47" s="54"/>
+      <c r="K47" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn, 2026-10-24: rotating soon. Update .env.playwright and the GitHub secrets (PLAYWRIGHT_TEST1_PASSWORD, SUPABASE_DEV_TEST2_PASSWORD) at the same time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="34" customHeight="1">
+      <c r="A48" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-44</t>
+        </is>
+      </c>
+      <c r="B48" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C48" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testing</t>
+        </is>
+      </c>
+      <c r="D48" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build spec 0067: get the e2e check green. It has failed on every PR since it was added on 2026-08-15.</t>
+        </is>
+      </c>
+      <c r="E48" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0067 (approved 2026-10-21)</t>
+        </is>
+      </c>
+      <c r="F48" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G48" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frontend + Tests + CI</t>
+        </is>
+      </c>
+      <c r="H48" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I48" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J48" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0067 approved</t>
+        </is>
+      </c>
+      <c r="K48" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Causes: the /beta Submit button moves 69px when the CAPTCHA finishes (a real visitor bug too), Early Adopters test checks a removed heading, CI never gets the test4@ login, vaccination tests can't seed data in CI (will be skipped there). Needs PA-45 for its last two checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="34" customHeight="1">
+      <c r="A49" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-45</t>
+        </is>
+      </c>
+      <c r="B49" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="C49" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testing</t>
+        </is>
+      </c>
+      <c r="D49" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Update the GitHub secrets the e2e job uses: re-enter PLAYWRIGHT_TEST3_ADMIN_EMAIL/PASSWORD and add PLAYWRIGHT_TEST4_SITTER_EMAIL/PASSWORD.</t>
+        </is>
+      </c>
+      <c r="E49" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0067 AC4/AC5</t>
+        </is>
+      </c>
+      <c r="F49" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G49" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dashboard</t>
+        </is>
+      </c>
+      <c r="H49" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I49" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J49" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0067</t>
+        </is>
+      </c>
+      <c r="K49" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Copy values from .env.playwright. GitHub &gt; repo &gt; Settings &gt; Secrets and variables &gt; Actions. Do it with PA-43 so CI gets the rotated passwords too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="34" customHeight="1">
+      <c r="A50" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-46</t>
+        </is>
+      </c>
+      <c r="B50" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C50" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testing</t>
+        </is>
+      </c>
+      <c r="D50" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cache Playwright's browsers in the CI e2e job, so a slow package server can't time it out.</t>
+        </is>
+      </c>
+      <c r="E50" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PR #22 CI run, 2026-10-23</t>
+        </is>
+      </c>
+      <c r="F50" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G50" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CI</t>
+        </is>
+      </c>
+      <c r="H50" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I50" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J50" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K50" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On PR #22 the job spent its full 20-minute limit downloading Ubuntu packages and was cancelled before any test ran. Not in 0067's scope; raise when 0067 is built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="34" customHeight="1">
+      <c r="A51" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-47</t>
+        </is>
+      </c>
+      <c r="B51" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C51" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testing</t>
+        </is>
+      </c>
+      <c r="D51" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Redo the abandoned PR #19/#20 work: the vaccination e2e test should refuse to run unless the CLI is linked to dev, and should clean up its test data even when a test fails.</t>
+        </is>
+      </c>
+      <c r="E51" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Closed PRs #19/#20 (built without spec review)</t>
+        </is>
+      </c>
+      <c r="F51" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G51" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tests</t>
+        </is>
+      </c>
+      <c r="H51" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I51" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J51" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K51" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Needs a new spec Lynn reviews first. Branches claude/cranky-ptolemy-795759 and claude/xenodochial-bell-d19ae3 are still on GitHub for reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="34" customHeight="1">
+      <c r="A52" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-48</t>
+        </is>
+      </c>
+      <c r="B52" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C52" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testing</t>
+        </is>
+      </c>
+      <c r="D52" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investigate e2e tests that fail only sometimes (check-in history on 09-01; bottom nav, home cards and pet editing on 08-19).</t>
+        </is>
+      </c>
+      <c r="E52" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0067 non-goal</t>
+        </is>
+      </c>
+      <c r="F52" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn (Claude Code)</t>
+        </is>
+      </c>
+      <c r="G52" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investigation</t>
+        </is>
+      </c>
+      <c r="H52" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I52" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J52" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K52" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Best done after PA-44, so real failures stand out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="34" customHeight="1">
+      <c r="A53" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA-49</t>
+        </is>
+      </c>
+      <c r="B53" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P2</t>
+        </is>
+      </c>
+      <c r="C53" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process</t>
+        </is>
+      </c>
+      <c r="D53" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decide whether to make e2e a required check once it has passed several runs in a row.</t>
+        </is>
+      </c>
+      <c r="E53" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0067 non-goal</t>
+        </is>
+      </c>
+      <c r="F53" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lynn</t>
+        </is>
+      </c>
+      <c r="G53" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decision</t>
+        </is>
+      </c>
+      <c r="H53" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not Started</t>
+        </is>
+      </c>
+      <c r="I53" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="J53" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not written</t>
+        </is>
+      </c>
+      <c r="K53" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Today only frontend and edge-functions are required. CLAUDE.md's 'trial through 9/3' note is part of PA-40.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K47"/>
+  <autoFilter ref="A4:K53"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B47">
+  <conditionalFormatting sqref="B5:B53">
     <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"P0"</formula>
     </cfRule>
@@ -12955,7 +13301,7 @@
       <formula>"P2"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H47">
+  <conditionalFormatting sqref="H5:H53">
     <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="Complete">
       <formula>NOT(ISERROR(SEARCH("Complete",H5)))</formula>
     </cfRule>
@@ -12966,7 +13312,7 @@
       <formula>NOT(ISERROR(SEARCH("Not Started",H5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I47">
+  <conditionalFormatting sqref="I5:I53">
     <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Mark PA-17 complete: bare domain redirects to www, prod CORS set
Lynn added a Cloudflare redirect rule (wyskerwatch.com/* -> www, 301),
confirmed live. Prod CORS_ALLOWED_ORIGINS now lists both www and the
bare domain as a safety net; all 4 public Edge Functions verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/Wysker_Watch_Launch_Plan.xlsx
+++ b/docs/planning/Wysker_Watch_Launch_Plan.xlsx
@@ -11469,7 +11469,7 @@
       </c>
       <c r="H21" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not Started</t>
+          <t xml:space="preserve">Complete</t>
         </is>
       </c>
       <c r="I21" s="56" t="inlineStr">
@@ -11479,12 +11479,12 @@
       </c>
       <c r="J21" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not written</t>
+          <t xml:space="preserve">Not needed (config + Cloudflare rule)</t>
         </is>
       </c>
       <c r="K21" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Still unset on prod. Three code comments disagree about which domain is canonical. Signup will fail for anyone arriving at the other domain unless it redirects. Lynn, 2026-10-24: www.wyskerwatch.com is the official address; wyskerwatch.com (no www) is also reachable and listed in Cloudflare. So: set CORS_ALLOWED_ORIGINS on prod to both, or add a Cloudflare redirect from the bare domain to www. Couldn't check from here whether a redirect already exists (Bot Fight Mode blocks automated requests).</t>
+          <t xml:space="preserve">Still unset on prod. Three code comments disagree about which domain is canonical. Signup will fail for anyone arriving at the other domain unless it redirects. Lynn, 2026-10-24: www.wyskerwatch.com is the official address; wyskerwatch.com (no www) is also reachable and listed in Cloudflare. So: set CORS_ALLOWED_ORIGINS on prod to both, or add a Cloudflare redirect from the bare domain to www. Couldn't check from here whether a redirect already exists (Bot Fight Mode blocks automated requests). DONE 2026-10-24: Lynn added a Cloudflare redirect rule ('Bare domain to www', 301, https://wyskerwatch.com/* -&gt; https://www.wyskerwatch.com/${1}), confirmed live. Prod CORS_ALLOWED_ORIGINS set to https://www.wyskerwatch.com,https://wyskerwatch.com as a safety net; all 4 public functions (beta-signup, early-adopter-signup, sign-up, confirm-email) verified accepting both and no longer accepting localhost. The 'three code comments disagree about the canonical domain' part is still open (www is canonical).</t>
         </is>
       </c>
     </row>

</xml_diff>